<commit_message>
NUOVI CAMBIAMENTI - cambiata questione ordinamento; predisposto tutto per il testing
</commit_message>
<xml_diff>
--- a/PS-VRP/Dati_output/Report_Problemi.xlsx
+++ b/PS-VRP/Dati_output/Report_Problemi.xlsx
@@ -7,9 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Problemi Lettura Excel" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Incompatibilità" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Veicoli errati" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Commesse su veicoli errati" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Problemi Lettura Excel" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +426,99 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P6"/>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>commessa</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>motivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>252417</v>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>nessuna compatibilità con alcuna macchina</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>252466</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>nessuna compatibilità con alcuna macchina</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>252980</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>nessuna compatibilità con alcuna macchina</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:P10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -530,27 +623,32 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>254225</v>
+        <v>251310</v>
       </c>
       <c r="B2" s="1" t="n">
-        <v>45975</v>
+        <v>45770</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>IN STAMPA</t>
+          <t>STAMPATO</t>
         </is>
       </c>
       <c r="D2" s="1" t="n">
-        <v>45960</v>
+        <v>45849</v>
       </c>
       <c r="E2" t="n">
         <v>6</v>
       </c>
       <c r="F2" t="n">
-        <v>3943</v>
+        <v>8611</v>
       </c>
       <c r="G2" t="n">
-        <v>200</v>
+        <v>336</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
@@ -558,10 +656,10 @@
         </is>
       </c>
       <c r="J2" t="n">
-        <v>60</v>
+        <v>410</v>
       </c>
       <c r="K2" t="n">
-        <v>780</v>
+        <v>820</v>
       </c>
       <c r="L2" s="2" t="n"/>
       <c r="M2" t="inlineStr">
@@ -570,43 +668,30 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>X</t>
-        </is>
-      </c>
-      <c r="P2" t="n">
-        <v>40635</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>233333</v>
-      </c>
-      <c r="B3" s="1" t="n">
-        <v>45972</v>
-      </c>
+        <v>251905</v>
+      </c>
+      <c r="B3" s="2" t="n"/>
       <c r="C3" t="inlineStr">
         <is>
-          <t>STAMPATO</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="n"/>
+          <t>IN STAMPA</t>
+        </is>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>45849</v>
+      </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F3" t="n">
-        <v>12</v>
+        <v>13841</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
-      </c>
-      <c r="H3" t="inlineStr">
-        <is>
-          <t>1</t>
-        </is>
+        <v>1000</v>
       </c>
       <c r="I3" t="inlineStr">
         <is>
@@ -614,12 +699,14 @@
         </is>
       </c>
       <c r="J3" t="n">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="K3" t="n">
-        <v>860</v>
-      </c>
-      <c r="L3" s="2" t="n"/>
+        <v>825</v>
+      </c>
+      <c r="L3" t="n">
+        <v>76</v>
+      </c>
       <c r="M3" t="inlineStr">
         <is>
           <t>Dati OK</t>
@@ -631,48 +718,44 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>253258</v>
+        <v>252453</v>
       </c>
       <c r="B4" s="1" t="n">
-        <v>45922</v>
+        <v>45845</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
           <t>STAMPATO</t>
         </is>
       </c>
-      <c r="D4" s="2" t="n"/>
+      <c r="D4" s="1" t="n">
+        <v>45849</v>
+      </c>
       <c r="E4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F4" t="n">
-        <v>4805</v>
+        <v>2990</v>
       </c>
       <c r="G4" t="n">
-        <v>223</v>
+        <v>169</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2</t>
-        </is>
-      </c>
-      <c r="I4" t="inlineStr">
-        <is>
-          <t>bobina</t>
-        </is>
-      </c>
+          <t>3 / 4</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="n"/>
       <c r="J4" t="n">
-        <v>250</v>
+        <v>190</v>
       </c>
       <c r="K4" t="n">
-        <v>1000</v>
-      </c>
-      <c r="L4" t="n">
-        <v>76</v>
-      </c>
+        <v>760</v>
+      </c>
+      <c r="L4" s="2" t="n"/>
       <c r="M4" t="inlineStr">
         <is>
-          <t>Dati OK</t>
+          <t xml:space="preserve"> ERR tipologia incarto non definita</t>
         </is>
       </c>
       <c r="N4" t="n">
@@ -681,55 +764,60 @@
     </row>
     <row r="5">
       <c r="A5" t="n">
-        <v>252459</v>
+        <v>252354</v>
       </c>
       <c r="B5" s="1" t="n">
-        <v>45855</v>
+        <v>45849</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>STAMPATO</t>
-        </is>
-      </c>
-      <c r="D5" s="2" t="n"/>
+          <t>IN STAMPA</t>
+        </is>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>45849</v>
+      </c>
       <c r="E5" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F5" t="n">
-        <v>4000</v>
+        <v>5060</v>
       </c>
       <c r="G5" t="n">
-        <v>91</v>
+        <v>100</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>foglio</t>
+          <t>bobina</t>
         </is>
       </c>
       <c r="J5" t="n">
-        <v>200</v>
+        <v>85</v>
       </c>
       <c r="K5" t="n">
-        <v>480</v>
-      </c>
-      <c r="L5" t="n">
-        <v>0</v>
-      </c>
+        <v>595</v>
+      </c>
+      <c r="L5" s="2" t="n"/>
       <c r="M5" t="inlineStr">
         <is>
           <t>Dati OK</t>
         </is>
       </c>
       <c r="N5" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="n">
-        <v>251310</v>
+        <v>251704</v>
       </c>
       <c r="B6" s="1" t="n">
-        <v>45770</v>
+        <v>45846</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -737,20 +825,20 @@
         </is>
       </c>
       <c r="D6" s="1" t="n">
-        <v>45769</v>
+        <v>45849</v>
       </c>
       <c r="E6" t="n">
-        <v>6</v>
+        <v>0</v>
       </c>
       <c r="F6" t="n">
-        <v>8611</v>
+        <v>28904</v>
       </c>
       <c r="G6" t="n">
-        <v>336</v>
+        <v>2217</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>6</t>
+          <t>1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -759,10 +847,10 @@
         </is>
       </c>
       <c r="J6" t="n">
-        <v>410</v>
+        <v>340</v>
       </c>
       <c r="K6" t="n">
-        <v>820</v>
+        <v>1020</v>
       </c>
       <c r="L6" s="2" t="n"/>
       <c r="M6" t="inlineStr">
@@ -773,86 +861,214 @@
       <c r="N6" t="n">
         <v>1</v>
       </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:D2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>nome</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>peso</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>zone</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>partenza</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>40629 (interno)</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P6" t="n">
+        <v>40054</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>252450</v>
+      </c>
+      <c r="B7" s="1" t="n">
+        <v>45852</v>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>IN STAMPA</t>
+        </is>
+      </c>
+      <c r="D7" s="1" t="n">
+        <v>45849</v>
+      </c>
+      <c r="E7" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>5718</v>
+      </c>
+      <c r="G7" t="n">
+        <v>300</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>6</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>bobina</t>
+        </is>
+      </c>
+      <c r="J7" t="n">
+        <v>390</v>
+      </c>
+      <c r="K7" t="n">
+        <v>780</v>
+      </c>
+      <c r="L7" s="2" t="n"/>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>Dati OK</t>
+        </is>
+      </c>
+      <c r="N7" t="n">
         <v>0</v>
       </c>
     </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:A2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>id</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="n">
-        <v>253940</v>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>252983</v>
+      </c>
+      <c r="B8" s="1" t="n">
+        <v>45847</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>IN STAMPA</t>
+        </is>
+      </c>
+      <c r="D8" s="1" t="n">
+        <v>45862</v>
+      </c>
+      <c r="E8" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" t="n">
+        <v>1912</v>
+      </c>
+      <c r="G8" t="n">
+        <v>97</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>bobina</t>
+        </is>
+      </c>
+      <c r="J8" t="n">
+        <v>85</v>
+      </c>
+      <c r="K8" t="n">
+        <v>425</v>
+      </c>
+      <c r="L8" s="2" t="n"/>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>Dati OK</t>
+        </is>
+      </c>
+      <c r="N8" t="n">
+        <v>4</v>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>X</t>
+        </is>
+      </c>
+      <c r="P8" t="n">
+        <v>40055</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>252666</v>
+      </c>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>DA STAMPARE</t>
+        </is>
+      </c>
+      <c r="D9" s="1" t="n">
+        <v>45901</v>
+      </c>
+      <c r="E9" t="n">
+        <v>6</v>
+      </c>
+      <c r="F9" t="n">
+        <v>13175</v>
+      </c>
+      <c r="G9" t="n">
+        <v>600</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>bobina</t>
+        </is>
+      </c>
+      <c r="J9" t="n">
+        <v>680</v>
+      </c>
+      <c r="K9" t="n">
+        <v>680</v>
+      </c>
+      <c r="L9" t="n">
+        <v>70</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>Dati OK</t>
+        </is>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>233333</v>
+      </c>
+      <c r="B10" s="1" t="n">
+        <v>45845</v>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>STAMPATO</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="n"/>
+      <c r="E10" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" t="n">
+        <v>12</v>
+      </c>
+      <c r="G10" t="n">
+        <v>1</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>bobina</t>
+        </is>
+      </c>
+      <c r="J10" t="n">
+        <v>169</v>
+      </c>
+      <c r="K10" t="n">
+        <v>860</v>
+      </c>
+      <c r="L10" s="2" t="n"/>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>Dati OK</t>
+        </is>
+      </c>
+      <c r="N10" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
EURISTICO BEST FIT + ALL'EURISTICO FINALE DOPO xGG
</commit_message>
<xml_diff>
--- a/PS-VRP/Dati_output/Report_Problemi.xlsx
+++ b/PS-VRP/Dati_output/Report_Problemi.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B4"/>
+  <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="25" customWidth="1" min="1" max="1"/>
@@ -447,7 +447,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>252417</v>
+        <v>254492</v>
       </c>
       <c r="B2" t="inlineStr">
         <is>
@@ -457,7 +457,7 @@
     </row>
     <row r="3">
       <c r="A3" t="n">
-        <v>252466</v>
+        <v>255579</v>
       </c>
       <c r="B3" t="inlineStr">
         <is>
@@ -467,9 +467,59 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>252980</v>
+        <v>255578</v>
       </c>
       <c r="B4" t="inlineStr">
+        <is>
+          <t>nessuna compatibilità con alcuna macchina</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>254830</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>nessuna compatibilità con alcuna macchina</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>255580</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>nessuna compatibilità con alcuna macchina</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>260242</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>nessuna compatibilità con alcuna macchina</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>260241</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>nessuna compatibilità con alcuna macchina</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>255452</v>
+      </c>
+      <c r="B9" t="inlineStr">
         <is>
           <t>nessuna compatibilità con alcuna macchina</t>
         </is>

</xml_diff>

<commit_message>
Versione per prova in azienda
</commit_message>
<xml_diff>
--- a/PS-VRP/Dati_output/Report_Problemi.xlsx
+++ b/PS-VRP/Dati_output/Report_Problemi.xlsx
@@ -7,10 +7,10 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Veicoli errati" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Commesse su veicoli errati" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Problemi Lettura Excel" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Incompatibilità" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Commesse su veicoli errati" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Problemi Lettura Excel" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Incompatibilità" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Veicoli errati" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -426,88 +426,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="25" customWidth="1" min="1" max="1"/>
-    <col width="25" customWidth="1" min="2" max="2"/>
-    <col width="25" customWidth="1" min="3" max="3"/>
-    <col width="25" customWidth="1" min="4" max="4"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>nome</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>peso</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>zone</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>partenza</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>40981 (interno)</t>
-        </is>
-      </c>
-      <c r="D2" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>40993 (interno)</t>
-        </is>
-      </c>
-      <c r="D3" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>40993 (interno)</t>
-        </is>
-      </c>
-      <c r="D4" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>41001 (interno)</t>
-        </is>
-      </c>
-      <c r="D5" t="n">
-        <v>0</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:A5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -523,7 +441,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>254635</v>
+        <v>243224</v>
       </c>
     </row>
     <row r="3">
@@ -533,7 +451,7 @@
     </row>
     <row r="4">
       <c r="A4" t="n">
-        <v>243224</v>
+        <v>254635</v>
       </c>
     </row>
     <row r="5">
@@ -546,7 +464,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -861,7 +779,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -969,4 +887,142 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="25" customWidth="1" min="1" max="1"/>
+    <col width="25" customWidth="1" min="2" max="2"/>
+    <col width="25" customWidth="1" min="3" max="3"/>
+    <col width="25" customWidth="1" min="4" max="4"/>
+    <col width="25" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>nome</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>capacita</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>zone</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>partenza</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>40981 (esterno)</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1" t="n">
+        <v>46037</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Creato automaticamente per commessa 254635.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>40993 (esterno)</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" s="1" t="n">
+        <v>46038</v>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Creato automaticamente per commessa 255481.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>40993 (esterno)</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>0</v>
+      </c>
+      <c r="D4" s="1" t="n">
+        <v>46034</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Creato automaticamente per commessa 243224.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>41001 (esterno)</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="1" t="n">
+        <v>46045</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Creato automaticamente per commessa 255504.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>41004 (esterno)</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="1" t="n">
+        <v>46034</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Creato automaticamente per commessa 255388.0</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>